<commit_message>
Card layout final + KMs rule
</commit_message>
<xml_diff>
--- a/samples/visit_log.xlsx
+++ b/samples/visit_log.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Raw Data" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Ignore Me" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Raw Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ignore Me" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,10 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="DD-MMM-YYYY"/>
-    <numFmt numFmtId="166" formatCode="HH:MM"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="DD-MMM-YYYY"/>
+    <numFmt numFmtId="165" formatCode="HH:MM"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -58,12 +57,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -429,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R23"/>
+  <dimension ref="A1:S23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -527,12 +528,17 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="Q3" s="2" t="inlineStr">
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>KMs</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
         <is>
           <t>VISITS</t>
         </is>
       </c>
-      <c r="R3" s="2" t="inlineStr">
+      <c r="S3" s="2" t="inlineStr">
         <is>
           <t>SOP Visit</t>
         </is>
@@ -549,7 +555,7 @@
           <t>AFZAL CHEEMA</t>
         </is>
       </c>
-      <c r="C4" s="3" t="n">
+      <c r="C4" s="5" t="n">
         <v>46296</v>
       </c>
       <c r="D4" t="inlineStr">
@@ -572,19 +578,19 @@
           <t>FSD-1</t>
         </is>
       </c>
-      <c r="H4" s="4" t="n">
+      <c r="H4" s="6" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="I4" s="4" t="n">
+      <c r="I4" s="6" t="n">
         <v>0.5</v>
       </c>
       <c r="J4" t="n">
         <v>4</v>
       </c>
-      <c r="K4" s="4" t="n">
+      <c r="K4" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="L4" s="4" t="n">
+      <c r="L4" s="6" t="n">
         <v>0.4375</v>
       </c>
       <c r="M4" t="n">
@@ -604,9 +610,11 @@
         </is>
       </c>
       <c r="Q4" t="n">
+        <v>80</v>
+      </c>
+      <c r="R4" t="n">
         <v>1</v>
       </c>
-      <c r="R4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -619,7 +627,7 @@
           <t>AFZAL CHEEMA</t>
         </is>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C5" s="5" t="n">
         <v>46296</v>
       </c>
       <c r="D5" t="inlineStr">
@@ -642,19 +650,19 @@
           <t>FSD-2</t>
         </is>
       </c>
-      <c r="H5" s="4" t="n">
+      <c r="H5" s="6" t="n">
         <v>0.5208333333333334</v>
       </c>
-      <c r="I5" s="4" t="n">
+      <c r="I5" s="6" t="n">
         <v>0.7083333333333334</v>
       </c>
       <c r="J5" t="n">
         <v>4.5</v>
       </c>
-      <c r="K5" s="4" t="n">
+      <c r="K5" s="6" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="L5" s="4" t="n">
+      <c r="L5" s="6" t="n">
         <v>0.625</v>
       </c>
       <c r="M5" t="n">
@@ -674,30 +682,13 @@
         </is>
       </c>
       <c r="Q5" t="n">
+        <v>65</v>
+      </c>
+      <c r="R5" t="n">
         <v>1</v>
       </c>
-      <c r="R5" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr"/>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
@@ -709,7 +700,7 @@
           <t>Afzaal Cheema</t>
         </is>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="C7" s="5" t="n">
         <v>46297</v>
       </c>
       <c r="D7" t="inlineStr">
@@ -732,19 +723,19 @@
           <t>FSD-1</t>
         </is>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="H7" s="6" t="n">
         <v>0.3541666666666667</v>
       </c>
-      <c r="I7" s="4" t="n">
+      <c r="I7" s="6" t="n">
         <v>0.6666666666666666</v>
       </c>
       <c r="J7" t="n">
         <v>7.5</v>
       </c>
-      <c r="K7" s="4" t="n">
+      <c r="K7" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="L7" s="4" t="n">
+      <c r="L7" s="6" t="n">
         <v>0.4791666666666667</v>
       </c>
       <c r="M7" t="n">
@@ -758,11 +749,12 @@
           <t>Market Visit</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr"/>
       <c r="Q7" t="n">
+        <v>110</v>
+      </c>
+      <c r="R7" t="n">
         <v>1</v>
       </c>
-      <c r="R7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -775,7 +767,7 @@
           <t>AFZAL CHEEMA</t>
         </is>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="C8" s="5" t="n">
         <v>46298</v>
       </c>
       <c r="D8" t="inlineStr">
@@ -798,19 +790,19 @@
           <t>FSD-3</t>
         </is>
       </c>
-      <c r="H8" s="4" t="n">
+      <c r="H8" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="I8" s="4" t="n">
+      <c r="I8" s="6" t="n">
         <v>0.5</v>
       </c>
       <c r="J8" t="n">
         <v>3</v>
       </c>
-      <c r="K8" s="4" t="n">
+      <c r="K8" s="6" t="n">
         <v>0.3854166666666667</v>
       </c>
-      <c r="L8" s="4" t="n">
+      <c r="L8" s="6" t="n">
         <v>0.4270833333333333</v>
       </c>
       <c r="M8" t="n">
@@ -829,10 +821,9 @@
           <t>Short day</t>
         </is>
       </c>
-      <c r="Q8" t="n">
+      <c r="R8" t="n">
         <v>1</v>
       </c>
-      <c r="R8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -845,7 +836,7 @@
           <t>AFZAL CHEEMA</t>
         </is>
       </c>
-      <c r="C9" s="3" t="n">
+      <c r="C9" s="5" t="n">
         <v>46299</v>
       </c>
       <c r="D9" t="inlineStr">
@@ -853,9 +844,6 @@
           <t>Sun</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
       <c r="O9" t="inlineStr">
         <is>
           <t>Leave</t>
@@ -866,8 +854,6 @@
           <t>Casual leave</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -880,7 +866,7 @@
           <t>AFZAL CHEEMA</t>
         </is>
       </c>
-      <c r="C10" s="3" t="n">
+      <c r="C10" s="5" t="n">
         <v>46300</v>
       </c>
       <c r="D10" t="inlineStr">
@@ -888,9 +874,6 @@
           <t>Mon</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
       <c r="O10" t="inlineStr">
         <is>
           <t>Meeting</t>
@@ -901,8 +884,6 @@
           <t>Monthly Meeting</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -915,7 +896,7 @@
           <t>AFZAL CHEEMA</t>
         </is>
       </c>
-      <c r="C11" s="3" t="n">
+      <c r="C11" s="5" t="n">
         <v>46301</v>
       </c>
       <c r="D11" t="inlineStr">
@@ -923,17 +904,11 @@
           <t>Tue</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
       <c r="O11" t="inlineStr">
         <is>
           <t>Officework</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -946,7 +921,7 @@
           <t>AFZAL CHEEMA</t>
         </is>
       </c>
-      <c r="C12" s="3" t="n">
+      <c r="C12" s="5" t="n">
         <v>46302</v>
       </c>
       <c r="D12" t="inlineStr">
@@ -954,9 +929,6 @@
           <t>Wed</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
       <c r="O12" t="inlineStr">
         <is>
           <t>Transit</t>
@@ -967,8 +939,9 @@
           <t>Travel to SGD</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
+      <c r="Q12" t="n">
+        <v>180</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -981,7 +954,7 @@
           <t>AFZAL CHEEMA</t>
         </is>
       </c>
-      <c r="C13" s="3" t="n">
+      <c r="C13" s="5" t="n">
         <v>46303</v>
       </c>
       <c r="D13" t="inlineStr">
@@ -1004,19 +977,19 @@
           <t>SGD-1</t>
         </is>
       </c>
-      <c r="H13" s="4" t="n">
+      <c r="H13" s="6" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="I13" s="4" t="n">
+      <c r="I13" s="6" t="n">
         <v>0.7083333333333334</v>
       </c>
       <c r="J13" t="n">
         <v>9</v>
       </c>
-      <c r="K13" s="4" t="n">
+      <c r="K13" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="L13" s="4" t="n">
+      <c r="L13" s="6" t="n">
         <v>0.5416666666666666</v>
       </c>
       <c r="M13" t="n">
@@ -1030,11 +1003,12 @@
           <t>Market Visit</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr"/>
       <c r="Q13" t="n">
+        <v>1250</v>
+      </c>
+      <c r="R13" t="n">
         <v>1</v>
       </c>
-      <c r="R13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1047,7 +1021,7 @@
           <t>Ahmed Khan</t>
         </is>
       </c>
-      <c r="C14" s="3" t="n">
+      <c r="C14" s="5" t="n">
         <v>46296</v>
       </c>
       <c r="D14" t="inlineStr">
@@ -1070,19 +1044,19 @@
           <t>LHR-1</t>
         </is>
       </c>
-      <c r="H14" s="4" t="n">
+      <c r="H14" s="6" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="I14" s="4" t="n">
+      <c r="I14" s="6" t="n">
         <v>0.6666666666666666</v>
       </c>
       <c r="J14" t="n">
         <v>8</v>
       </c>
-      <c r="K14" s="4" t="n">
+      <c r="K14" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="L14" s="4" t="n">
+      <c r="L14" s="6" t="n">
         <v>0.5</v>
       </c>
       <c r="M14" t="n">
@@ -1096,11 +1070,12 @@
           <t>Market Visit</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr"/>
       <c r="Q14" t="n">
+        <v>90</v>
+      </c>
+      <c r="R14" t="n">
         <v>1</v>
       </c>
-      <c r="R14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1113,7 +1088,7 @@
           <t>Ahmed Khan</t>
         </is>
       </c>
-      <c r="C15" s="3" t="n">
+      <c r="C15" s="5" t="n">
         <v>46297</v>
       </c>
       <c r="D15" t="inlineStr">
@@ -1121,17 +1096,11 @@
           <t>Fri</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
       <c r="O15" t="inlineStr">
         <is>
           <t>Leave</t>
         </is>
       </c>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1144,7 +1113,7 @@
           <t>Ahmed Khan</t>
         </is>
       </c>
-      <c r="C16" s="3" t="n">
+      <c r="C16" s="5" t="n">
         <v>46298</v>
       </c>
       <c r="D16" t="inlineStr">
@@ -1152,9 +1121,6 @@
           <t>Sat</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
       <c r="O16" t="inlineStr">
         <is>
           <t>Meeting</t>
@@ -1165,8 +1131,6 @@
           <t>Region meeting</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1179,7 +1143,7 @@
           <t>Sara Malik</t>
         </is>
       </c>
-      <c r="C17" s="3" t="n">
+      <c r="C17" s="5" t="n">
         <v>46296</v>
       </c>
       <c r="D17" t="inlineStr">
@@ -1202,19 +1166,19 @@
           <t>KHI-1</t>
         </is>
       </c>
-      <c r="H17" s="4" t="n">
+      <c r="H17" s="6" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="I17" s="4" t="n">
+      <c r="I17" s="6" t="n">
         <v>0.625</v>
       </c>
       <c r="J17" t="n">
         <v>7</v>
       </c>
-      <c r="K17" s="4" t="n">
+      <c r="K17" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="L17" s="4" t="n">
+      <c r="L17" s="6" t="n">
         <v>0.4666666666666667</v>
       </c>
       <c r="M17" t="n">
@@ -1228,11 +1192,12 @@
           <t>Market Visit</t>
         </is>
       </c>
-      <c r="P17" t="inlineStr"/>
       <c r="Q17" t="n">
+        <v>70</v>
+      </c>
+      <c r="R17" t="n">
         <v>1</v>
       </c>
-      <c r="R17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1245,7 +1210,7 @@
           <t>Sara Malik</t>
         </is>
       </c>
-      <c r="C18" s="3" t="n">
+      <c r="C18" s="5" t="n">
         <v>46297</v>
       </c>
       <c r="D18" t="inlineStr">
@@ -1253,17 +1218,11 @@
           <t>Fri</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
       <c r="O18" t="inlineStr">
         <is>
           <t>Officework</t>
         </is>
       </c>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1276,7 +1235,7 @@
           <t>Sara Malik</t>
         </is>
       </c>
-      <c r="C19" s="3" t="n">
+      <c r="C19" s="5" t="n">
         <v>46298</v>
       </c>
       <c r="D19" t="inlineStr">
@@ -1299,19 +1258,19 @@
           <t>KHI-1</t>
         </is>
       </c>
-      <c r="H19" s="4" t="n">
+      <c r="H19" s="6" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="I19" s="4" t="n">
+      <c r="I19" s="6" t="n">
         <v>0.5</v>
       </c>
       <c r="J19" t="n">
         <v>4</v>
       </c>
-      <c r="K19" s="4" t="n">
+      <c r="K19" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="L19" s="4" t="n">
+      <c r="L19" s="6" t="n">
         <v>0.4166666666666667</v>
       </c>
       <c r="M19" t="n">
@@ -1325,11 +1284,12 @@
           <t>Market Visit</t>
         </is>
       </c>
-      <c r="P19" t="inlineStr"/>
       <c r="Q19" t="n">
+        <v>55</v>
+      </c>
+      <c r="R19" t="n">
         <v>1</v>
       </c>
-      <c r="R19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1342,7 +1302,7 @@
           <t>Sara Malik</t>
         </is>
       </c>
-      <c r="C20" s="3" t="n">
+      <c r="C20" s="5" t="n">
         <v>46298</v>
       </c>
       <c r="D20" t="inlineStr">
@@ -1365,19 +1325,19 @@
           <t>KHI-2</t>
         </is>
       </c>
-      <c r="H20" s="4" t="n">
+      <c r="H20" s="6" t="n">
         <v>0.5208333333333334</v>
       </c>
-      <c r="I20" s="4" t="n">
+      <c r="I20" s="6" t="n">
         <v>0.7083333333333334</v>
       </c>
       <c r="J20" t="n">
         <v>4.5</v>
       </c>
-      <c r="K20" s="4" t="n">
+      <c r="K20" s="6" t="n">
         <v>0.5416666666666666</v>
       </c>
-      <c r="L20" s="4" t="n">
+      <c r="L20" s="6" t="n">
         <v>0.5833333333333334</v>
       </c>
       <c r="M20" t="n">
@@ -1391,11 +1351,9 @@
           <t>Market Visit</t>
         </is>
       </c>
-      <c r="P20" t="inlineStr"/>
-      <c r="Q20" t="n">
+      <c r="R20" t="n">
         <v>1</v>
       </c>
-      <c r="R20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1408,7 +1366,7 @@
           <t>Unknown Person</t>
         </is>
       </c>
-      <c r="C21" s="3" t="n">
+      <c r="C21" s="5" t="n">
         <v>46304</v>
       </c>
       <c r="D21" t="inlineStr">
@@ -1431,19 +1389,19 @@
           <t>FSD-1</t>
         </is>
       </c>
-      <c r="H21" s="4" t="n">
+      <c r="H21" s="6" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="I21" s="4" t="n">
+      <c r="I21" s="6" t="n">
         <v>0.6666666666666666</v>
       </c>
       <c r="J21" t="n">
         <v>8</v>
       </c>
-      <c r="K21" s="4" t="n">
+      <c r="K21" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="L21" s="4" t="n">
+      <c r="L21" s="6" t="n">
         <v>0.5</v>
       </c>
       <c r="M21" t="n">
@@ -1463,9 +1421,11 @@
         </is>
       </c>
       <c r="Q21" t="n">
+        <v>40</v>
+      </c>
+      <c r="R21" t="n">
         <v>1</v>
       </c>
-      <c r="R21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1478,7 +1438,7 @@
           <t>Ahmed Khan</t>
         </is>
       </c>
-      <c r="C22" s="3" t="n">
+      <c r="C22" s="5" t="n">
         <v>46305</v>
       </c>
       <c r="D22" t="inlineStr">
@@ -1501,16 +1461,16 @@
           <t>LHR-2</t>
         </is>
       </c>
-      <c r="H22" s="4" t="n">
+      <c r="H22" s="6" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="I22" s="4" t="n">
+      <c r="I22" s="6" t="n">
         <v>0.375</v>
       </c>
-      <c r="K22" s="4" t="n">
+      <c r="K22" s="6" t="n">
         <v>0.6875</v>
       </c>
-      <c r="L22" s="4" t="n">
+      <c r="L22" s="6" t="n">
         <v>0.4166666666666667</v>
       </c>
       <c r="O22" t="inlineStr">
@@ -1524,9 +1484,11 @@
         </is>
       </c>
       <c r="Q22" t="n">
+        <v>12</v>
+      </c>
+      <c r="R22" t="n">
         <v>1</v>
       </c>
-      <c r="R22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1534,29 +1496,15 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
       <c r="J23" t="n">
         <v>40</v>
       </c>
-      <c r="K23" t="inlineStr"/>
-      <c r="L23" t="inlineStr"/>
       <c r="M23" t="n">
         <v>20</v>
       </c>
       <c r="N23" t="n">
         <v>20</v>
       </c>
-      <c r="O23" t="inlineStr"/>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>